<commit_message>
LDA reducer, grid-line removal, re-segmentation, resumable CNN baseline
- Reducer chosen on training data only (LDA beat PCA in train CV)
- Interior vertical grid-line removal in preprocessing
- Recognition-guided re-segmentation for flagged lines, segmentation evaluation
- CNN baseline: epoch cap raised to 300, sleep-corrected timing,
  per-epoch checkpoints so long points can run over several nights
- Devanagari for all 57 labels and a verification sheet
- Results of the LDA learning curve, ablation and CNN points 72-250
</commit_message>
<xml_diff>
--- a/docs/01_literature_survey/Literature_Survey_30_Papers.xlsx
+++ b/docs/01_literature_survey/Literature_Survey_30_Papers.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\sem5\Ds\cp\modi-lipi-xai\docs\01_literature_survey\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03747728-4638-4188-8B51-0D3B63C84A3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B4500C3-7AB2-4954-828A-3790B37FF7EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="642" uniqueCount="435">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="628" uniqueCount="421">
   <si>
     <t>No</t>
   </si>
@@ -1296,48 +1296,6 @@
   </si>
   <si>
     <t>Papers 4, 6, 14 and 18.</t>
-  </si>
-  <si>
-    <t>How this survey was compiled</t>
-  </si>
-  <si>
-    <t>The 30 papers are the open-access PDFs in docs/03_reference_papers/ (downloaded 2026-10-12). Each row was filled in from the paper's own text (abstract, method, results and conclusion sections). Titles, authors, venues and DOIs come from the OpenAlex index and arXiv.</t>
-  </si>
-  <si>
-    <t>Things to check before submitting</t>
-  </si>
-  <si>
-    <t>1. Author names and venues were taken from an index, not typed from each PDF. Check them against the papers before they go into a reference list.</t>
-  </si>
-  <si>
-    <t>2. 'Best reported (%)' is the single headline figure for each experimental paper, with the metric named beside it. Where a paper gives both validation and test accuracy, or contradicts itself, the 'Results as stated' and 'Limitations' columns say so.</t>
-  </si>
-  <si>
-    <t>3. These 30 papers are the ones that could be downloaded legally. Several stronger papers are paywalled (Springer / IEEE) and are NOT in this survey, including the Zernike + DCT (2023), HOG-based (2024) and wavelet + SVD (2020) papers. They are listed at the end of docs/03_reference_papers/INDEX.md.</t>
-  </si>
-  <si>
-    <t>4. Eight rows are review or theoretical papers and four are not recognition papers (CAPTCHA, font design, tools, Unicode proposal). A stricter survey would replace some of them.</t>
-  </si>
-  <si>
-    <t>Observations worth raising in the report</t>
-  </si>
-  <si>
-    <t>- Papers 4, 6, 14 and 18 report the same baseline CNN figures (train 91.12%, validation 87.25%). Papers 4 and 18 also share the same VGG16 training accuracy (97.62%).</t>
-  </si>
-  <si>
-    <t>- Papers 4, 6 and 19 give different accuracy figures in their abstract or conclusion than in their results section.</t>
-  </si>
-  <si>
-    <t>- Paper 7 reports 45.08% validation accuracy next to 97.38% test accuracy for the same model; paper 11 reports validation accuracy 13 points above training accuracy.</t>
-  </si>
-  <si>
-    <t>- The public benchmark used by papers 4, 6, 14 and 18 has 46 classes x 90 images = 4,140 images. This is the small-data regime the project's learning curve starts from.</t>
-  </si>
-  <si>
-    <t>Column guide</t>
-  </si>
-  <si>
-    <t>Paper type: Experimental / Review / Conceptual / Tool / Standard.   Approach: what kind of model the paper's own experiments use.   The last three content columns record evidence for the project's research gaps.</t>
   </si>
 </sst>
 </file>
@@ -4296,74 +4254,46 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A1" s="13" t="s">
-        <v>421</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" ht="25" x14ac:dyDescent="0.35">
-      <c r="A2" s="14" t="s">
-        <v>422</v>
-      </c>
+      <c r="A1" s="13"/>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A2" s="14"/>
     </row>
     <row r="3" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="13" t="s">
-        <v>423</v>
-      </c>
+      <c r="A3" s="13"/>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A4" s="14" t="s">
-        <v>424</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" ht="25" x14ac:dyDescent="0.35">
-      <c r="A5" s="14" t="s">
-        <v>425</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" ht="37.5" x14ac:dyDescent="0.35">
-      <c r="A6" s="14" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" ht="25" x14ac:dyDescent="0.35">
-      <c r="A7" s="14" t="s">
-        <v>427</v>
-      </c>
+      <c r="A4" s="14"/>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A5" s="14"/>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A6" s="14"/>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A7" s="14"/>
     </row>
     <row r="8" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A8" s="13" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" ht="25" x14ac:dyDescent="0.35">
-      <c r="A9" s="14" t="s">
-        <v>429</v>
-      </c>
+      <c r="A8" s="13"/>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A9" s="14"/>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A10" s="14" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" ht="25" x14ac:dyDescent="0.35">
-      <c r="A11" s="14" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" ht="25" x14ac:dyDescent="0.35">
-      <c r="A12" s="14" t="s">
-        <v>432</v>
-      </c>
+      <c r="A10" s="14"/>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A11" s="14"/>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A12" s="14"/>
     </row>
     <row r="13" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A13" s="13" t="s">
-        <v>433</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" ht="25" x14ac:dyDescent="0.35">
-      <c r="A14" s="14" t="s">
-        <v>434</v>
-      </c>
+      <c r="A13" s="13"/>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A14" s="14"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Base papers sheet, rewritten synopsis objectives, leave-one-out ablation
Literature survey gets a second sheet with the 8 base papers: why each was chosen, what we take from it, what we do differently and which objective it supports. Synopsis objectives rewritten around those papers; outdated lines (Streamlit, Plotly, PCA wording) corrected. Objective 2 asks how much each descriptor adds, so the ablation now also drops one family at a time (HOG+LBP, HOG+Zernike, Zernike+LBP).
</commit_message>
<xml_diff>
--- a/docs/01_literature_survey/Literature_Survey_30_Papers.xlsx
+++ b/docs/01_literature_survey/Literature_Survey_30_Papers.xlsx
@@ -3,9 +3,11 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
     <sheet name="Literature Survey" sheetId="1" r:id="rId1"/>
+    <sheet name="Base Papers" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Literature Survey'!$A$1:$P$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Base Papers'!$A$1:$J$9</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -2563,4 +2565,473 @@
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" paperSize="9" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="9" customWidth="1"/>
+    <col min="2" max="2" width="40" customWidth="1"/>
+    <col min="3" max="3" width="11" customWidth="1"/>
+    <col min="4" max="4" width="26" customWidth="1"/>
+    <col min="5" max="5" width="30" customWidth="1"/>
+    <col min="6" max="6" width="44" customWidth="1"/>
+    <col min="7" max="7" width="40" customWidth="1"/>
+    <col min="8" max="8" width="50" customWidth="1"/>
+    <col min="9" max="9" width="18" customWidth="1"/>
+    <col min="10" max="10" width="40" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="36" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sr No (in survey)</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Name of paper</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Year of publication</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Name of author</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Journal/Conference Name</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Why it is a base paper</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">What we take from it</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">What we do differently (gap we address)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Related objective</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drive Link for the Research Paper</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="150" customHeight="1">
+      <c r="A2" s="3">
+        <v>4</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Handwritten Modi Script Character Recognition Using CNN and VGG16 Algorithms</t>
+        </is>
+      </c>
+      <c r="C2" s="3">
+        <v>2025</v>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mrunali Manohar Bhong, Prof. Nanda Kulkarni</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">International Journal of Advanced Research in Science Communication and Technology</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Uses the standard public benchmark (46 classes, 90 images each) that most Modi papers report on, and compares a plain CNN with VGG16.</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The benchmark size (about 72 training images per class) is our smallest learning-curve point, and its CNN results are our deep-learning reference.</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Their VGG16 shows an 8-point gap between training and validation accuracy. We measure how much data a CNN actually needs, on a fixed test set, instead of reporting one number.</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Objective 1, Objective 5</t>
+        </is>
+      </c>
+      <c r="J2" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://drive.google.com/file/d/1MVf2DNKJMDea1oef1b630xe91zuuPy4S/view?usp=drive_link</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="150" customHeight="1">
+      <c r="A3" s="3">
+        <v>6</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Modi Script Character Recognition Using Convolutional Neural Networks and Attention-Based CNN Architecture</t>
+        </is>
+      </c>
+      <c r="C3" s="3">
+        <v>2025</v>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shweta Kolte, Dr. Brijendra Gupta</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">International Journal of Advanced Research in Science Communication and Technology</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The strongest recent CNN result on the same benchmark, and it names visually similar characters as the main difficulty.</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The idea that the hard part of Modi is telling look-alike characters apart.</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">They describe confused characters but never list them. We list the most confused pairs and use SHAP to show which part of the character separates them.</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Objective 4</t>
+        </is>
+      </c>
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://drive.google.com/file/d/1NZ3rY-qkA8b1TcicNiu0BjBTLWwEj1aM/view?usp=drive_link</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="150" customHeight="1">
+      <c r="A4" s="3">
+        <v>7</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Modi Script Handwritten Character Classification using Drop-out Induced Incremental Learning Approach</t>
+        </is>
+      </c>
+      <c r="C4" s="3">
+        <v>2025</v>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chaitali Chandankhede</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Journal of Information Systems Engineering &amp; Management</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Clear published example of deep models overfitting on small Modi data (97% test vs 45% validation, about 21 images per class).</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Motivation for checking data size before trusting deep-learning accuracy on Modi.</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We keep a single fixed test set and nested training sets, so every accuracy we report is on images the model never saw.</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Objective 5</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://drive.google.com/file/d/1U7zROdFpBjG0FY2Cwzm5rczjE79BnuB-/view?usp=drive_link</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="150" customHeight="1">
+      <c r="A5" s="3">
+        <v>14</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Offline MODI script character recognition using deep learning techniques</t>
+        </is>
+      </c>
+      <c r="C5" s="3">
+        <v>2024</v>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sakshi  Mandke, Varsha Pimprale, Prakash Date</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Library Progress (International)</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The only paper that compares classical models (KNN, SVM) and deep models (CNN, VGG16, ResNet) on the same Modi data.</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The classical-versus-deep comparison itself.</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Their KNN and SVM were given raw pixels, so they had no real chance (75% and 77%). We give the classical models proper handcrafted features and compare at several data sizes.</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Objective 2, Objective 5</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://drive.google.com/file/d/1RWlQ9FzKuy8_4o90BnGnJfzd00b5r9Bx/view?usp=drive_link</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="150" customHeight="1">
+      <c r="A6" s="3">
+        <v>21</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implementing a Hybrid Deep Learning Approach to Achieve Classic Handwritten Alphanumeric MODI Recognition</t>
+        </is>
+      </c>
+      <c r="C6" s="3">
+        <v>2022</v>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Maitreyi Ekbote, Aishwary Jadhav, Dayanand D. Ambawade</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">International Journal of Engineering and Advanced Technology</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Closest prior work: it uses Random Forest and XGBoost for Modi characters and numerals.</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Random Forest and XGBoost as classifiers.</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">They used VGG16 features (not explainable) and each classifier on its own. We use handcrafted features, combine RF, SVM and XGBoost in a stacking ensemble, and explain every prediction with SHAP.</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Objective 3, Objective 4</t>
+        </is>
+      </c>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://drive.google.com/file/d/1qXUwvijQoq5t8v2GfDWO3HT7S6EInmi2/view?usp=drive_link</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="150" customHeight="1">
+      <c r="A7" s="3">
+        <v>24</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">An Experimental Exploration of Segmentation Techniques for Modi Script</t>
+        </is>
+      </c>
+      <c r="C7" s="3">
+        <v>2019</v>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bhumika Solanki, Maya Ingle</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">International Journal of Computer Applications</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Compares segmentation methods (edge detection vs K-means) on Modi images.</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cleaning and separating the character from the background before recognition.</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">It works only on single isolated characters. Our app also splits a line of separated characters into individual characters in reading order.</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Objective 6</t>
+        </is>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://drive.google.com/file/d/1RBR1pdz762jXLJpUxWNKjcxLFLml24w1/view?usp=drive_link</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="150" customHeight="1">
+      <c r="A8" s="3">
+        <v>26</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">An Approach for Recognizing Modi Lipi using Ostu's Binarization Algorithm and Kohenen Neural Network</t>
+        </is>
+      </c>
+      <c r="C8" s="3">
+        <v>2015</v>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sidra Anam, Saurabh Gupta</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">International Journal of Computer Applications</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Early Modi recogniser that uses Otsu binarisation, and reports that similar-shaped characters perform worst.</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Otsu binarisation as the main preprocessing step.</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">They used 22 characters with 8 images each and raw pixels. We use all 57 classes, a public dataset and handcrafted descriptors.</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Objective 1, Objective 4</t>
+        </is>
+      </c>
+      <c r="J8" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://drive.google.com/file/d/1QXS084xRD2H1IKdQHM_8haOl41oQI_RI/view?usp=drive_link</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="150" customHeight="1">
+      <c r="A9" s="3">
+        <v>28</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Recognition of Handwritten MODI Numerals using Hu and Zernike features</t>
+        </is>
+      </c>
+      <c r="C9" s="3">
+        <v>2014</v>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sadanand A. Kulkarni, Prashant L. Borde, Ramesh R. Manza, Pravin L. Yannawar</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">arXiv preprint (1404.1151)</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shows that Zernike moments describe Modi shapes better than Hu moments (86.7% vs 70%).</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Zernike moments as one of our three descriptors.</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">They tested only 100 digit images with a distance classifier. We fuse Zernike with HOG and LBP on all 57 classes and run an ablation to see what each adds.</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Objective 2</t>
+        </is>
+      </c>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://drive.google.com/file/d/15-3xfLp2ngTmFOScLksUdC8gKVkXtDZt/view?usp=drive_link</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:J9"/>
+  <hyperlinks>
+    <hyperlink ref="J2" r:id="rId1"/>
+    <hyperlink ref="J3" r:id="rId2"/>
+    <hyperlink ref="J4" r:id="rId3"/>
+    <hyperlink ref="J5" r:id="rId4"/>
+    <hyperlink ref="J6" r:id="rId5"/>
+    <hyperlink ref="J7" r:id="rId6"/>
+    <hyperlink ref="J8" r:id="rId7"/>
+    <hyperlink ref="J9" r:id="rId8"/>
+  </hyperlinks>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToWidth="1" fitToHeight="0"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Four objectives from the base papers, simpler synopsis, literature review deck
Synopsis rewritten in plain language with four objectives tied to 7 base papers; the Scope section and extra bullets removed. Base Papers sheet updated to match. Added Literature_Review_Presentation.pptx (18 slides, every paper linked to its PDF on Drive). README now reports the leave-one-out ablation.
</commit_message>
<xml_diff>
--- a/docs/01_literature_survey/Literature_Survey_30_Papers.xlsx
+++ b/docs/01_literature_survey/Literature_Survey_30_Papers.xlsx
@@ -7,7 +7,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Literature Survey'!$A$1:$P$31</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Base Papers'!$A$1:$J$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Base Papers'!$A$1:$J$8</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -2674,7 +2674,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Objective 1, Objective 5</t>
+          <t xml:space="preserve">Objective 4</t>
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr">
@@ -2722,7 +2722,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Objective 4</t>
+          <t xml:space="preserve">Objective 3</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
@@ -2770,7 +2770,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Objective 5</t>
+          <t xml:space="preserve">Objective 4</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
@@ -2818,7 +2818,7 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Objective 2, Objective 5</t>
+          <t xml:space="preserve">Objective 1, Objective 4</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
@@ -2866,7 +2866,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Objective 3, Objective 4</t>
+          <t xml:space="preserve">Objective 2</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
@@ -2877,19 +2877,19 @@
     </row>
     <row r="7" ht="150" customHeight="1">
       <c r="A7" s="3">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">An Experimental Exploration of Segmentation Techniques for Modi Script</t>
+          <t xml:space="preserve">An Approach for Recognizing Modi Lipi using Ostu's Binarization Algorithm and Kohenen Neural Network</t>
         </is>
       </c>
       <c r="C7" s="3">
-        <v>2019</v>
+        <v>2015</v>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bhumika Solanki, Maya Ingle</t>
+          <t xml:space="preserve">Sidra Anam, Saurabh Gupta</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -2899,128 +2899,80 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Compares segmentation methods (edge detection vs K-means) on Modi images.</t>
+          <t xml:space="preserve">Early Modi recogniser that uses Otsu binarisation, and reports that similar-shaped characters perform worst.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cleaning and separating the character from the background before recognition.</t>
+          <t xml:space="preserve">Otsu binarisation as the main preprocessing step.</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">It works only on single isolated characters. Our app also splits a line of separated characters into individual characters in reading order.</t>
+          <t xml:space="preserve">They used 22 characters with 8 images each and raw pixels. We use all 57 classes, a public dataset and handcrafted descriptors.</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Objective 6</t>
+          <t xml:space="preserve">Objective 1, Objective 3</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://drive.google.com/file/d/1RBR1pdz762jXLJpUxWNKjcxLFLml24w1/view?usp=drive_link</t>
+          <t xml:space="preserve">https://drive.google.com/file/d/1QXS084xRD2H1IKdQHM_8haOl41oQI_RI/view?usp=drive_link</t>
         </is>
       </c>
     </row>
     <row r="8" ht="150" customHeight="1">
       <c r="A8" s="3">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">An Approach for Recognizing Modi Lipi using Ostu's Binarization Algorithm and Kohenen Neural Network</t>
+          <t xml:space="preserve">Recognition of Handwritten MODI Numerals using Hu and Zernike features</t>
         </is>
       </c>
       <c r="C8" s="3">
-        <v>2015</v>
+        <v>2014</v>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sidra Anam, Saurabh Gupta</t>
+          <t xml:space="preserve">Sadanand A. Kulkarni, Prashant L. Borde, Ramesh R. Manza, Pravin L. Yannawar</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">International Journal of Computer Applications</t>
+          <t xml:space="preserve">arXiv preprint (1404.1151)</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Early Modi recogniser that uses Otsu binarisation, and reports that similar-shaped characters perform worst.</t>
+          <t xml:space="preserve">Shows that Zernike moments describe Modi shapes better than Hu moments (86.7% vs 70%).</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Otsu binarisation as the main preprocessing step.</t>
+          <t xml:space="preserve">Zernike moments as one of our three descriptors.</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">They used 22 characters with 8 images each and raw pixels. We use all 57 classes, a public dataset and handcrafted descriptors.</t>
+          <t xml:space="preserve">They tested only 100 digit images with a distance classifier. We fuse Zernike with HOG and LBP on all 57 classes and run an ablation to see what each adds.</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Objective 1, Objective 4</t>
+          <t xml:space="preserve">Objective 1</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://drive.google.com/file/d/1QXS084xRD2H1IKdQHM_8haOl41oQI_RI/view?usp=drive_link</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="150" customHeight="1">
-      <c r="A9" s="3">
-        <v>28</v>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Recognition of Handwritten MODI Numerals using Hu and Zernike features</t>
-        </is>
-      </c>
-      <c r="C9" s="3">
-        <v>2014</v>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Sadanand A. Kulkarni, Prashant L. Borde, Ramesh R. Manza, Pravin L. Yannawar</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">arXiv preprint (1404.1151)</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Shows that Zernike moments describe Modi shapes better than Hu moments (86.7% vs 70%).</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Zernike moments as one of our three descriptors.</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">They tested only 100 digit images with a distance classifier. We fuse Zernike with HOG and LBP on all 57 classes and run an ablation to see what each adds.</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Objective 2</t>
-        </is>
-      </c>
-      <c r="J9" s="4" t="inlineStr">
-        <is>
           <t xml:space="preserve">https://drive.google.com/file/d/15-3xfLp2ngTmFOScLksUdC8gKVkXtDZt/view?usp=drive_link</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J9"/>
+  <autoFilter ref="A1:J8"/>
   <hyperlinks>
     <hyperlink ref="J2" r:id="rId1"/>
     <hyperlink ref="J3" r:id="rId2"/>
@@ -3029,7 +2981,6 @@
     <hyperlink ref="J6" r:id="rId5"/>
     <hyperlink ref="J7" r:id="rId6"/>
     <hyperlink ref="J8" r:id="rId7"/>
-    <hyperlink ref="J9" r:id="rId8"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" paperSize="9" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
Literature survey sheet rewritten in plain student language
Problem statement, methodology, application, limitation, objective, finding, challenge and research gap columns rewritten for all 30 papers, plus the Base Papers sheet. Facts, datasets and numbers unchanged.
</commit_message>
<xml_diff>
--- a/docs/01_literature_survey/Literature_Survey_30_Papers.xlsx
+++ b/docs/01_literature_survey/Literature_Survey_30_Papers.xlsx
@@ -212,12 +212,12 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text CAPTCHAs in Latin script are increasingly broken by OCR and machine learning. The paper asks whether the cursive, conjunct-heavy Modi script can make CAPTCHAs harder for machines while staying solvable by people.</t>
+          <t xml:space="preserve">Normal text CAPTCHAs are getting easy for bots to break. The author asks if Modi, which computers find hard to read, could be used to make CAPTCHAs that people can solve but bots can't.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Character generation with warping, distortion and noise (obfuscator module). CAPTCHA generation framework; tested against humans and OCR/ML attacks.</t>
+          <t xml:space="preserve">Generates Modi words and letters as images and distorts them (warping, noise). The plan is to test them on people and on OCR attacks.</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -227,7 +227,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Web security (CAPTCHA for websites); cultural promotion of Modi script</t>
+          <t xml:space="preserve">CAPTCHAs on websites, and making more people aware of Modi</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -237,27 +237,27 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No quantitative evaluation, no dataset, no attack model details.</t>
+          <t xml:space="preserve">There are no numbers at all, no dataset and no details on how the attacks were tested.</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Design a framework that generates Modi-script CAPTCHAs and evaluates their usability and robustness against automated attacks.</t>
+          <t xml:space="preserve">To design a system that makes Modi CAPTCHAs and checks how easy they are for people and how hard they are for bots.</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Modi-based CAPTCHAs are reported to have a much lower automated-attack success rate than Latin or Devanagari CAPTCHAs (qualitative claim, no numbers).</t>
+          <t xml:space="preserve">The author says bots succeed less often on Modi CAPTCHAs than on English or Devanagari ones, but doesn't give any figures.</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Balancing human readability against machine resistance; Modi's complexity that helps security is the same thing that makes recognition hard.</t>
+          <t xml:space="preserve">The CAPTCHA has to stay readable for people while being hard for machines.</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No dataset, no numeric evaluation and no attack model. Indirectly confirms that automatic Modi recognition is still unsolved.</t>
+          <t xml:space="preserve">Nothing is actually measured. It mainly tells us that reading Modi automatically is still an open problem.</t>
         </is>
       </c>
       <c r="P2" s="4" t="inlineStr">
@@ -290,12 +290,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Large Modi archives cannot be read because there is no reliable automatic transliteration into Devanagari, and Modi is a low-resource script.</t>
+          <t xml:space="preserve">Lots of old Modi documents can't be read because there is no good tool to convert Modi into Devanagari, and Modi doesn't have much data to train on.</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sequence encoding of sentences. Encoder-decoder with stacked LSTM (512 hidden units), sentence level.</t>
+          <t xml:space="preserve">An encoder-decoder model with stacked LSTM layers that converts whole Modi sentences into Devanagari.</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -305,7 +305,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Digitising and transliterating historical Modi documents into Devanagari</t>
+          <t xml:space="preserve">Converting Modi documents into Devanagari so more people can read them</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -315,27 +315,27 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Several accuracy figures (85.16%, 86.12%, 97.16%) are reported without a clear definition of how they differ. Corpus availability not stated.</t>
+          <t xml:space="preserve">They give several accuracy numbers (85.16%, 86.12%, 97.16%) without clearly saying how each was measured, and the corpus doesn't seem to be public.</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Build a sentence-level Modi-to-Devanagari transliteration model that handles variable-length sequences.</t>
+          <t xml:space="preserve">To build a model that converts Modi sentences into Devanagari, even when sentences are of different lengths.</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">A stacked-LSTM encoder-decoder reaches BLEU 46, 85.16% character accuracy and 86.12% word accuracy (CER 0.09).</t>
+          <t xml:space="preserve">The model gets a BLEU score of 46, 85.16% of characters right and 86.12% of words right.</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Long-range context, variable sentence lengths, scarce parallel data.</t>
+          <t xml:space="preserve">Long sentences of different lengths, and not much parallel data to learn from.</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Works on text sequences, not on handwritten images; depends on an upstream character recogniser. Accuracy figures are not clearly defined and the corpus is not public. No explainability.</t>
+          <t xml:space="preserve">It works on typed text, not handwriting, so it needs a character recogniser before it. It also doesn't explain its output.</t>
         </is>
       </c>
       <c r="P3" s="4" t="inlineStr">
@@ -368,12 +368,12 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hundreds of thousands of Modi documents sit unread in archives because very few people can read the script.</t>
+          <t xml:space="preserve">Thousands of Modi documents are stuck in archives because hardly anyone can read them.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Planned: image clean-up, character segmentation. Proposed 5-stage 'ModiAnuwad' pipeline: preprocessing, segmentation, CNN recognition, Transformer translation to English, grammar correction.</t>
+          <t xml:space="preserve">Proposes a 5-step system called ModiAnuwad: clean the image, cut out characters, recognise them with a CNN, translate with a Transformer, then fix grammar.</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -383,7 +383,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">End-to-end Modi document to English translation for historians and archives</t>
+          <t xml:space="preserve">Translating Modi documents into English for historians and archives</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -393,27 +393,27 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Purely conceptual; no dataset, no implementation, no evaluation.</t>
+          <t xml:space="preserve">It's only a plan. There's no dataset, no code and no results.</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Propose ModiAnuwad, a five-stage pipeline: clean-up, segmentation, CNN recognition, Transformer translation and grammar correction.</t>
+          <t xml:space="preserve">To design a full pipeline that turns a Modi document image into English text.</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Only a system design is presented; no experiments were run.</t>
+          <t xml:space="preserve">Only the design is presented; nothing was built or tested.</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Every stage (segmentation, recognition, translation) is itself an open problem for Modi.</t>
+          <t xml:space="preserve">Every step in the pipeline (cutting characters, recognising them, translating) is still unsolved for Modi.</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Purely conceptual: no dataset, implementation or evaluation. The recognition stage it relies on is what needs solving first.</t>
+          <t xml:space="preserve">The recognition step it depends on is exactly the part that needs to be solved first.</t>
         </is>
       </c>
       <c r="P4" s="4" t="inlineStr">
@@ -446,12 +446,12 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Handwritten Modi characters are hard to recognise because of writer variation, noise and visually similar cursive shapes.</t>
+          <t xml:space="preserve">Handwritten Modi letters are hard to recognise because everyone writes differently and many letters look alike.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Noise removal, resizing (200x200 / 224x224), binarisation, segmentation, augmentation (rotation, zoom, shift, flip). Custom CNN and VGG16 (ImageNet transfer learning).</t>
+          <t xml:space="preserve">Cleans and resizes the images, adds rotated and shifted copies, then trains a small CNN and a pre-trained VGG16.</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -461,7 +461,7 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Digital preservation of Modi manuscripts; character-level OCR</t>
+          <t xml:space="preserve">Recognising single Modi letters for digitising manuscripts</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -471,27 +471,27 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">8-point train/validation gap for VGG16 on 90 images per class (overfitting). Conclusion (94.3%) contradicts the results section (89.50%). No per-class analysis.</t>
+          <t xml:space="preserve">VGG16 scores 8 points higher on training data than on validation data, so it is overfitting. The conclusion says 94.3% but the results table says 89.5%. There's no per-letter analysis.</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Compare a custom CNN with transfer-learned VGG16 on public and self-collected handwritten Modi data (46 classes).</t>
+          <t xml:space="preserve">To compare a simple CNN with VGG16 on the public 46-letter Modi dataset and on their own handwriting samples.</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">VGG16 beats the plain CNN (89.50% vs 87.25% validation), especially on similar-looking characters.</t>
+          <t xml:space="preserve">VGG16 did better than the plain CNN (89.5% vs 87.25% on validation), especially on letters that look alike.</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Small data (90 images per class) causes overfitting; similar-looking characters.</t>
+          <t xml:space="preserve">Only 90 images per letter, which isn't much for deep learning.</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">8-point train/validation gap shows overfitting on small data; conclusion and results disagree (94.3% vs 89.5%). No per-class or confusion analysis, no explainability, no classical baseline with handcrafted features.</t>
+          <t xml:space="preserve">No list of which letters get confused, no explanation of predictions, and no proper classical model to compare against.</t>
         </is>
       </c>
       <c r="P5" s="4" t="inlineStr">
@@ -524,12 +524,12 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">About 40 million Modi documents are untransliterated, and prior work focuses on isolated characters rather than whole documents.</t>
+          <t xml:space="preserve">Around 40 million Modi documents haven't been transliterated, and most earlier work only looks at single letters, not full documents.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Document images from three historical eras. MoScNet: vision-language model with knowledge distillation (student has 163x fewer parameters than teacher).</t>
+          <t xml:space="preserve">Builds a dataset of 2,043 document images with Devanagari text, and a vision-language model (MoScNet) where a small student model learns from a big teacher model.</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -539,7 +539,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Direct document-level transliteration of Modi into Devanagari</t>
+          <t xml:space="preserve">Converting whole Modi documents into Devanagari</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -549,27 +549,27 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Document-level only, no character-level labels. Large model, needs GPU. arXiv preprint.</t>
+          <t xml:space="preserve">There are no letter-level labels, the models need a GPU, and it's still an arXiv preprint.</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Release the MoDeTrans dataset (2,043 document images) and a vision-language model (MoScNet) for direct transliteration.</t>
+          <t xml:space="preserve">To release a public document-level dataset and a model that reads a Modi page straight into Devanagari.</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">A distilled student model with 163x fewer parameters outperforms its teacher (BLEU 51.03) and is competitive on OCR benchmarks.</t>
+          <t xml:space="preserve">The small student model actually beats the teacher (BLEU 51.03) while being 163 times smaller.</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Degraded historical documents, three historical writing eras, very large models.</t>
+          <t xml:space="preserve">Old, damaged documents from three different periods, and very large models.</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No character-level labels or analysis; needs GPU-scale models; arXiv preprint. Not interpretable. Useful mainly as a source of real Modi document images.</t>
+          <t xml:space="preserve">It can't tell you which letters it got wrong or why. For us it's mainly a source of real Modi document images.</t>
         </is>
       </c>
       <c r="P6" s="4" t="inlineStr">
@@ -602,12 +602,12 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Plain CNNs confuse Modi characters that share most of their strokes.</t>
+          <t xml:space="preserve">Normal CNNs mix up Modi letters that share most of their strokes.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Resize to 224x224, normalisation. Baseline CNN vs attention-based CNN (spatial + channel attention).</t>
+          <t xml:space="preserve">Resizes images to 224 x 224 and compares a basic CNN with a CNN that has spatial and channel attention.</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -617,7 +617,7 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Handwritten Modi character recognition for digitisation</t>
+          <t xml:space="preserve">Recognising handwritten Modi letters</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
@@ -627,27 +627,27 @@
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Abstract and conclusion disagree (94.60% vs about 90%). Baseline CNN figures are identical to papers 4, 14 and 18. Confusing pairs are discussed but not tabulated.</t>
+          <t xml:space="preserve">The abstract says 94.60% but the conclusion says about 90%. The basic CNN numbers are the same as in papers 4, 14 and 18. Confused letters are talked about but never listed.</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Add spatial and channel attention to a CNN so it focuses on the strokes that distinguish similar characters.</t>
+          <t xml:space="preserve">To add attention to a CNN so it focuses on the strokes that separate similar letters.</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Attention CNN reported at 94.60% validation accuracy vs 87.25% for the baseline CNN.</t>
+          <t xml:space="preserve">The attention model is reported at 94.60% validation accuracy, against 87.25% for the basic CNN.</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">High visual similarity between characters; cursive style variation.</t>
+          <t xml:space="preserve">Letters that look very similar, and different writing styles.</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Abstract (94.6%) and conclusion (about 90%) disagree; baseline numbers repeat other papers. Confusing pairs are discussed but never tabulated, and attention maps are not used as explanations.</t>
+          <t xml:space="preserve">No table of which letters get confused, and the attention maps aren't used to explain anything.</t>
         </is>
       </c>
       <c r="P7" s="4" t="inlineStr">
@@ -680,12 +680,12 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Modi texts hold valuable knowledge (healthcare, food, Ayurveda) but the full character set including vowel combinations (barakhadi) has not been addressed.</t>
+          <t xml:space="preserve">Modi books on health, food and Ayurveda are hard to read, and no one had tried the full set of letter-plus-vowel combinations (barakhadi).</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Otsu, Sauvola and To-zero binarisation; augmentation; dropout. ResNet152, InceptionV3, InceptionResNetV2 with dropout; incremental learning (characters, then words).</t>
+          <t xml:space="preserve">Tries different ways of making the image black and white (Otsu, Sauvola, To-zero), adds dropout, and trains ResNet152, InceptionV3 and InceptionResNetV2 in stages (letters first, then words).</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -695,7 +695,7 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Recognition of the full Modi barakhadi (360 classes)</t>
+          <t xml:space="preserve">Recognising all 360 Modi barakhadi classes</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -705,27 +705,27 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Severe overfitting reported by the authors. Validation accuracy (45%) and test accuracy (97%) are far apart, which is not explained. About 21 training images per class.</t>
+          <t xml:space="preserve">The authors admit the model overfits badly. Validation accuracy (45%) and test accuracy (97%) are very far apart and this isn't explained. There are only about 21 training images per class.</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Classify 360 Modi character classes with deep CNNs, dropout and incremental learning (characters, then words).</t>
+          <t xml:space="preserve">To classify all 360 Modi character classes using deep CNNs with dropout and incremental learning.</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ResNet152 with To-zero binarisation reports 97.38% average test accuracy, but only 45.08% validation accuracy.</t>
+          <t xml:space="preserve">ResNet152 with To-zero thresholding reports 97.38% average test accuracy but only 45.08% on validation.</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Very few images per class (about 21) for 360 classes; severe overfitting.</t>
+          <t xml:space="preserve">Very few images for each of the 360 classes.</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Validation (45%) and test (97%) accuracies contradict each other without explanation; private data. A clear example of deep models overfitting on small Modi data.</t>
+          <t xml:space="preserve">A clear example of deep models overfitting on small Modi data. The two accuracy numbers can't both be right.</t>
         </is>
       </c>
       <c r="P8" s="4" t="inlineStr">
@@ -758,12 +758,12 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Modi recognition is hindered by intricate shapes, handwriting diversity and lack of datasets; deep-learning methods need to be reviewed together.</t>
+          <t xml:space="preserve">Modi letters are complex, people write them differently and there isn't much data, so the authors review how deep learning has been used for it.</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Literature review. Surveys template matching, feature extraction, CNN, transfer learning, CNN-SVM hybrids, GAN augmentation.</t>
+          <t xml:space="preserve">Literature review of template matching, CNNs, transfer learning, CNN with SVM, and GAN-based data augmentation.</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -773,7 +773,7 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Literature review for Modi OCR research</t>
+          <t xml:space="preserve">Background reading for Modi OCR research</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
@@ -783,27 +783,27 @@
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Narrative review. Several cited figures are not traceable to named datasets.</t>
+          <t xml:space="preserve">It's a narrative review, and some numbers it quotes can't be traced back to a dataset.</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Review CNN, transfer learning (VGG16, ResNet) and CNN-SVM hybrid approaches for Modi recognition.</t>
+          <t xml:space="preserve">To review the deep learning methods used for Modi recognition and their weak points.</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reported accuracies range from about 65% to over 90%; dataset scarcity and handwriting variation are the main obstacles.</t>
+          <t xml:space="preserve">Earlier work reports from about 65% to over 90%. Lack of data and different handwriting styles are the main problems.</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Comparing methods evaluated on different, often private datasets.</t>
+          <t xml:space="preserve">Comparing methods that were tested on different, often private, datasets.</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Narrative review; several cited figures cannot be traced to a named dataset. Explainability is only mentioned.</t>
+          <t xml:space="preserve">Explainability is mentioned but nothing is done with it.</t>
         </is>
       </c>
       <c r="P9" s="4" t="inlineStr">
@@ -836,12 +836,12 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Modi is harder to decipher than other scripts, and the many proposed techniques have not been surveyed together.</t>
+          <t xml:space="preserve">Modi is harder to read than most scripts and many methods have been tried, but they haven't been put together in one place.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Literature review. Surveys OCR, CNN, ANN, SVM, chain code, Zernike moments.</t>
+          <t xml:space="preserve">Literature review of OCR, CNN, ANN, SVM, chain code and Zernike moment methods.</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -861,27 +861,27 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Narrative; no comparison on a common dataset.</t>
+          <t xml:space="preserve">It doesn't compare the methods on the same data.</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Survey OCR, CNN, ANN, SVM, chain-code and Zernike-moment approaches for Modi.</t>
+          <t xml:space="preserve">To survey the techniques used for Modi character recognition.</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Deep learning dominates recent work; classical features such as Zernike moments appear in earlier studies.</t>
+          <t xml:space="preserve">Recent work is mostly deep learning; older work used shape features like Zernike moments.</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No common benchmark to compare methods fairly.</t>
+          <t xml:space="preserve">There is no common dataset to compare methods fairly.</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No comparison on a common dataset; handcrafted descriptors are listed but never fused or compared under one protocol.</t>
+          <t xml:space="preserve">Handcrafted features are listed, but no one combines them or tests them side by side.</t>
         </is>
       </c>
       <c r="P10" s="4" t="inlineStr">
@@ -914,12 +914,12 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Modi's connected, cursive characters and the lack of annotated data limit both traditional image processing and machine-learning OCR.</t>
+          <t xml:space="preserve">Modi letters are joined and cursive and there's little labelled data, which makes both simple image processing and machine learning struggle.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Literature review. Surveys thresholding, edge detection, CNN, transfer learning, CNN-SVM hybrids.</t>
+          <t xml:space="preserve">Systematic review with a comparison table of thresholding, edge detection, CNNs, transfer learning and CNN-SVM hybrids.</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -929,7 +929,7 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Review of Modi character recognition to guide future OCR work</t>
+          <t xml:space="preserve">Review to guide future Modi OCR work</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
@@ -939,27 +939,27 @@
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Compares numbers obtained on different datasets as if comparable.</t>
+          <t xml:space="preserve">It compares numbers from different datasets as if they were the same test.</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Systematically review advances and challenges, with a comparison table of prior methods.</t>
+          <t xml:space="preserve">To review what has worked and what hasn't in Modi character recognition.</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Deep models report the highest accuracies (ResNet50 94.55%, InceptionV3 93.92%) while traditional thresholding/edge methods had limited success.</t>
+          <t xml:space="preserve">Deep models report the highest numbers (ResNet50 94.55%, InceptionV3 93.92%), while simple thresholding methods did poorly.</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Limited annotated datasets and high style variability.</t>
+          <t xml:space="preserve">Few labelled datasets and lots of variation in handwriting.</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Compares accuracies from different datasets as if comparable; no study of how much data each approach needs.</t>
+          <t xml:space="preserve">Nobody looks at how much data each method needs.</t>
         </is>
       </c>
       <c r="P11" s="4" t="inlineStr">
@@ -992,12 +992,12 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Modi is unfamiliar to modern readers, and it is unclear which deep architecture works best for its characters.</t>
+          <t xml:space="preserve">Modi is unfamiliar to people today, and it's not clear which deep network works best for its letters.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Standard transfer-learning preprocessing. ResNet101, InceptionV3, Xception (transfer learning).</t>
+          <t xml:space="preserve">Transfer learning with three ImageNet models: ResNet101, InceptionV3 and Xception.</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -1007,7 +1007,7 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Handwritten Modi character classification</t>
+          <t xml:space="preserve">Recognising handwritten Modi letters</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -1017,27 +1017,27 @@
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dataset size and class count unclear. ResNet101's validation accuracy is 13 points above its training accuracy, which is unusual and unexplained. Conclusion names Xception best although ResNet101 has the higher validation score.</t>
+          <t xml:space="preserve">The dataset size and number of classes aren't clear. ResNet101 scores 13 points higher on validation than on training, which is strange and not explained. The conclusion picks Xception even though ResNet101 scored higher.</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Compare ResNet101, InceptionV3 and Xception with transfer learning.</t>
+          <t xml:space="preserve">To compare three pre-trained deep networks on Modi letters.</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ResNet101 reaches 90.36% validation, Xception 85.94%, InceptionV3 80.99%.</t>
+          <t xml:space="preserve">ResNet101 reached 90.36% on validation, Xception 85.94% and InceptionV3 80.99%.</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Small dataset; choosing among large pretrained models.</t>
+          <t xml:space="preserve">Small dataset and choosing between big pre-trained models.</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dataset size and classes not stated; ResNet101 validation is 13 points above training, unexplained; conclusion contradicts the numbers. Unstable rankings on small data.</t>
+          <t xml:space="preserve">Rankings of deep models look unstable when there's so little data.</t>
         </is>
       </c>
       <c r="P12" s="4" t="inlineStr">
@@ -1070,12 +1070,12 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transliterating handwritten Modi into Devanagari is hard because documents are complex and there is no standard dataset.</t>
+          <t xml:space="preserve">Converting handwritten Modi into Devanagari is hard because the documents are complex and there's no standard dataset.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Line images with Unicode ground truth; annotation tool. CRNN-based Calamari OCR (fine-tuned).</t>
+          <t xml:space="preserve">Builds 4,334 line images with Devanagari text and fine-tunes Calamari OCR, which is a CRNN model.</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1085,7 +1085,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Line-level transliteration of Modi manuscripts</t>
+          <t xml:space="preserve">Converting Modi manuscript lines into Devanagari</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
@@ -1095,27 +1095,27 @@
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Word-level accuracy is only 61%. Dataset not public. No standard benchmark exists.</t>
+          <t xml:space="preserve">Only 61% of whole words come out right, and the dataset isn't public.</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Treat transliteration as pattern recognition and fine-tune a CRNN (Calamari OCR) on Modi text lines.</t>
+          <t xml:space="preserve">To treat Modi-to-Devanagari conversion as a pattern recognition problem at the line level.</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">88.14% character-level and 61% whole-word accuracy on 845 test lines.</t>
+          <t xml:space="preserve">88.14% of characters are correct but only 61% of whole words.</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No standard dataset; connected writing without word boundaries.</t>
+          <t xml:space="preserve">No standard dataset, and words run together with no spaces.</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Word-level accuracy is low (61%); dataset not public; no error or confusion analysis.</t>
+          <t xml:space="preserve">No analysis of which errors happen most.</t>
         </is>
       </c>
       <c r="P13" s="4" t="inlineStr">
@@ -1148,12 +1148,12 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Modi characters are cursive, continuous and strikingly similar; documents lack word boundaries and suffer skew, noise and overlapping lines.</t>
+          <t xml:space="preserve">Modi letters are cursive and look alike, and documents have no word breaks, tilted lines and overlapping text.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Synthetic text-line images; Gaussian blur. LSTM network (ModiDev_LSTM_Model).</t>
+          <t xml:space="preserve">Generates Modi text from a font (with vowels, signs and joint letters), slightly tilts and blurs it, and trains an LSTM.</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -1163,7 +1163,7 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transcription of Modi documents into Devanagari</t>
+          <t xml:space="preserve">Transcribing Modi documents into Devanagari</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -1173,27 +1173,27 @@
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Synthetic (font-rendered) data only; limited to low-resolution images. Not validated on real handwriting.</t>
+          <t xml:space="preserve">All the data is generated from a font, so it was never tested on real handwriting.</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Build a synthetic Modi dataset with diacritics and conjuncts and an LSTM transcription model.</t>
+          <t xml:space="preserve">To build a synthetic Modi dataset and an LSTM model that handles vowel signs and joint letters.</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">94.67% character accuracy on synthetic test data, with an error breakdown by diacritic type.</t>
+          <t xml:space="preserve">94.67% character accuracy on the generated test data, with a breakdown of which vowel signs it gets wrong.</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Segmentation of continuous script; lack of real annotated data.</t>
+          <t xml:space="preserve">Splitting continuous writing and the lack of real labelled data.</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Synthetic, font-rendered data only; not validated on real handwriting. One of few papers with an error-type analysis.</t>
+          <t xml:space="preserve">One of the few papers that looks at error types, but only on font data.</t>
         </is>
       </c>
       <c r="P14" s="4" t="inlineStr">
@@ -1226,12 +1226,12 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Limited Modi datasets and many similar characters reduce recognition accuracy.</t>
+          <t xml:space="preserve">There isn't much Modi data and many letters look similar, which pulls accuracy down.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Augmentation. KNN, SVM, CNN, VGG16, ResNet compared.</t>
+          <t xml:space="preserve">Trains KNN, SVM, CNN, VGG16 and ResNet on the same augmented dataset and compares them.</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -1241,7 +1241,7 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Offline Modi character recognition</t>
+          <t xml:space="preserve">Recognising handwritten Modi letters</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
@@ -1251,27 +1251,27 @@
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Classical models are run without handcrafted features (features not described), so they are weak baselines. Parts of the text repeat figures from other papers.</t>
+          <t xml:space="preserve">KNN and SVM were given raw pixels with no proper features, so they never had a fair chance. The class count changes between 46 and 48 in the text.</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Compare KNN, SVM, CNN, VGG16 and ResNet on the same Modi dataset.</t>
+          <t xml:space="preserve">To compare classical and deep models on the same Modi data.</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">CNN 96% vs ResNet 87%, VGG16 85%, SVM 77%, KNN 75%.</t>
+          <t xml:space="preserve">CNN got 96%, ResNet 87%, VGG16 85%, SVM 77% and KNN 75%.</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Distinguishing similar characters with little data.</t>
+          <t xml:space="preserve">Telling similar letters apart with a small dataset.</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">KNN/SVM run without described handcrafted features, so the classical baseline is weak; class count inconsistent (46/48). Motivates a proper classical pipeline with fused descriptors.</t>
+          <t xml:space="preserve">The classical models had no handcrafted features, so the comparison is unfair to them. This is the main gap our project picks up.</t>
         </is>
       </c>
       <c r="P15" s="4" t="inlineStr">
@@ -1304,12 +1304,12 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Handwritten Modi documents must be converted to Devanagari for them to be accessible today.</t>
+          <t xml:space="preserve">Handwritten Modi has to be converted to Devanagari before people today can use it.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Describes data collection for a Modi dataset. Character recognition model plus rule-based Modi-to-Devanagari mapping.</t>
+          <t xml:space="preserve">A character recognition model followed by a rule-based mapping from Modi to Devanagari letters.</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -1319,7 +1319,7 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Modi-to-Devanagari character mapping for digitisation</t>
+          <t xml:space="preserve">Mapping Modi letters to Devanagari for digitisation</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
@@ -1329,27 +1329,27 @@
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No accuracy figures or dataset details.</t>
+          <t xml:space="preserve">No accuracy numbers or dataset details are given.</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Recognise handwritten Modi characters and map them to Devanagari with a conversion algorithm.</t>
+          <t xml:space="preserve">To recognise handwritten Modi letters and convert them to Devanagari.</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Claims accurate recognition and conversion across handwriting styles, but gives no numbers.</t>
+          <t xml:space="preserve">The authors say it works across handwriting styles but don't give any numbers.</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Handwriting style diversity; building a dataset.</t>
+          <t xml:space="preserve">Many different handwriting styles, and building a dataset.</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No accuracy figures, dataset details or evaluation protocol.</t>
+          <t xml:space="preserve">Without any evaluation, there's no way to check how well it works.</t>
         </is>
       </c>
       <c r="P16" s="4" t="inlineStr">
@@ -1382,12 +1382,12 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Many surveys on Modi recognition exist; their trends and gaps have not been consolidated.</t>
+          <t xml:space="preserve">There are already several reviews on Modi recognition, but nobody had put their findings together.</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Literature review. Surveys deep learning, transfer learning, thresholding.</t>
+          <t xml:space="preserve">Review of earlier reviews covering deep learning, transfer learning and thresholding.</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -1397,7 +1397,7 @@
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Meta-review of Modi recognition research</t>
+          <t xml:space="preserve">Summary of Modi recognition research</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
@@ -1407,27 +1407,27 @@
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Overlaps heavily with paper 10 (same cited figures).</t>
+          <t xml:space="preserve">It mostly repeats the same numbers as paper 10.</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Review existing literature surveys to identify methods, trends and open challenges.</t>
+          <t xml:space="preserve">To pull together trends and open problems from earlier reviews.</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Deep and transfer learning dominate; reported results include ResNet50 94.55% and a 95,000-image GSC + minimum-distance system at 83.19%.</t>
+          <t xml:space="preserve">Deep and transfer learning dominate. It also mentions a private 95,000-image, 55-class dataset with 83.19% accuracy.</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fragmented, non-comparable prior work.</t>
+          <t xml:space="preserve">Earlier work can't really be compared.</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Repeats figures from earlier reviews; no new analysis.</t>
+          <t xml:space="preserve">No new analysis or experiments.</t>
         </is>
       </c>
       <c r="P17" s="4" t="inlineStr">
@@ -1460,12 +1460,12 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Recognition performance depends on the size and variety of training images, and Modi lacks good datasets.</t>
+          <t xml:space="preserve">How well a recogniser works depends a lot on the training images, and Modi doesn't have a good dataset.</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Segmentation, augmentation, synthetic generation; 256x256 images; 10-fold cross-validation. Enhanced RNN, convolutional autoencoder, LSTM, GAN, DBN.</t>
+          <t xml:space="preserve">Collects 5,245 letters from 120 writers (46 classes), uses augmentation and synthetic images, and compares RNN, autoencoder, LSTM, GAN and DBN models with 10-fold cross-validation.</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -1475,7 +1475,7 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dataset creation for Modi handwritten character recognition</t>
+          <t xml:space="preserve">Building datasets for Modi letter recognition</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
@@ -1485,27 +1485,27 @@
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dataset not public. Results are modest and rounded to whole percentages.</t>
+          <t xml:space="preserve">The dataset isn't public and the results are rounded to whole numbers.</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Collect a 46-class Modi dataset (5,245 characters, 120 writers) and compare augmentation and synthetic-generation techniques with several models.</t>
+          <t xml:space="preserve">To compare different ways of building and enlarging a Modi image dataset.</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Enhanced RNN, convolutional autoencoder and GAN reach about 88%; LSTM 82%; DBN 72%.</t>
+          <t xml:space="preserve">The best models (enhanced RNN, autoencoder, GAN) reached about 88%; LSTM got 82% and DBN 72%.</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Collecting diverse handwriting; generating realistic synthetic samples.</t>
+          <t xml:space="preserve">Getting enough handwriting variety and making realistic synthetic images.</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dataset not public; modest, rounded results; no study of how accuracy grows with data size.</t>
+          <t xml:space="preserve">Doesn't check how accuracy changes as the amount of data grows.</t>
         </is>
       </c>
       <c r="P18" s="4" t="inlineStr">
@@ -1538,12 +1538,12 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">MODI character identification is complex, and a recogniser must work on both printed and handwritten scans.</t>
+          <t xml:space="preserve">Identifying Modi letters is complicated, and a system should work on both printed and handwritten scans.</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Segmentation, binarisation. CNN and VGG16.</t>
+          <t xml:space="preserve">Segments and binarises the scans, then trains a CNN and VGG16 on 48 letters.</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Modi character recognition from scanned papers</t>
+          <t xml:space="preserve">Recognising Modi letters from scanned pages</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
@@ -1563,27 +1563,27 @@
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Only training accuracy is given for VGG16. Figures are identical to paper 4 (same journal, two years later).</t>
+          <t xml:space="preserve">Only training accuracy is given for VGG16, and the numbers are the same as paper 4.</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Recognise 48 Modi characters with a CNN and VGG16.</t>
+          <t xml:space="preserve">To recognise printed and handwritten Modi letters with a CNN and VGG16.</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">CNN 87.25% validation; VGG16 97.62% training accuracy (validation not given).</t>
+          <t xml:space="preserve">The CNN got 87.25% on validation; VGG16 got 97.62% on training data (no validation number).</t>
         </is>
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Varying paper quality; similar characters.</t>
+          <t xml:space="preserve">Scans of different quality and look-alike letters.</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Only training accuracy for VGG16; figures identical to paper 4. No error analysis or explainability.</t>
+          <t xml:space="preserve">No error analysis and no explanations.</t>
         </is>
       </c>
       <c r="P19" s="4" t="inlineStr">
@@ -1616,12 +1616,12 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Modi's structure makes character recognition hard and no image database exists.</t>
+          <t xml:space="preserve">Modi letters are hard to recognise and there's no proper image database.</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Augmentation (flipping, noise). CNN.</t>
+          <t xml:space="preserve">Makes more training images by flipping and adding noise, then trains a CNN.</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -1631,7 +1631,7 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Handwritten Modi character recognition</t>
+          <t xml:space="preserve">Recognising handwritten Modi letters</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
@@ -1641,27 +1641,27 @@
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Abstract and results disagree (91.62% vs 96.58%). Dataset size and classes not given.</t>
+          <t xml:space="preserve">The abstract says 91.62% and the results say 96.58%. The dataset size and classes aren't given.</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Train a CNN on a Modi dataset enlarged with data augmentation.</t>
+          <t xml:space="preserve">To train a CNN on a small Modi dataset made bigger with augmentation.</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">91.62% accuracy in the abstract; 96.58% test accuracy in the results section.</t>
+          <t xml:space="preserve">Test accuracy is reported as 96.58% (91.62% in the abstract).</t>
         </is>
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tiny original dataset.</t>
+          <t xml:space="preserve">A very small starting dataset.</t>
         </is>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Abstract and results disagree; dataset size and class count not given; no comparison with other methods.</t>
+          <t xml:space="preserve">No comparison with other methods, and the two numbers don't match.</t>
         </is>
       </c>
       <c r="P20" s="4" t="inlineStr">
@@ -1694,12 +1694,12 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Millions of Modi documents remain unexplored and methods from 2010 to 2022 have not been compared systematically.</t>
+          <t xml:space="preserve">Millions of Modi documents are unread, and the methods from 2010 to 2022 hadn't been compared properly.</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Literature review. Compares feature-extraction and classification methods.</t>
+          <t xml:space="preserve">Systematic review comparing the features and classifiers used for Modi between 2010 and 2022.</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -1709,7 +1709,7 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Systematic review for choosing Modi recognition techniques</t>
+          <t xml:space="preserve">Helping choose a Modi recognition method</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
@@ -1719,27 +1719,27 @@
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The highest cited figures come from different, mostly private datasets.</t>
+          <t xml:space="preserve">The highest numbers it quotes come from different, mostly private datasets.</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Review and compare feature-extraction and classification methods for Modi (2010-2022).</t>
+          <t xml:space="preserve">To review and compare the methods used for Modi recognition.</t>
         </is>
       </c>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Concludes CNN is best, citing up to 99.78% accuracy.</t>
+          <t xml:space="preserve">Concludes that CNNs work best, quoting up to 99.78% accuracy.</t>
         </is>
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Results come from different, mostly private datasets.</t>
+          <t xml:space="preserve">Results come from datasets that can't be compared.</t>
         </is>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Highest figures are not comparable across datasets; no controlled classical-vs-deep comparison at equal data sizes.</t>
+          <t xml:space="preserve">No fair comparison of classical and deep methods at the same data size.</t>
         </is>
       </c>
       <c r="P21" s="4" t="inlineStr">
@@ -1772,12 +1772,12 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No quality Modi database or literature exists, making recognition of characters and numerals difficult.</t>
+          <t xml:space="preserve">There's no good Modi database and not much literature, which makes recognising letters and numerals hard.</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">VGG16 as feature extractor. VGG16 features classified by Random Forest and XGBoost.</t>
+          <t xml:space="preserve">Uses VGG16 to extract features and then classifies them with Random Forest and XGBoost.</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -1787,7 +1787,7 @@
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Recognition of Modi characters and numerals</t>
+          <t xml:space="preserve">Recognising Modi letters and numerals</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
@@ -1797,27 +1797,27 @@
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Features are learned (VGG16), not handcrafted, so the model is not interpretable. Each classifier used alone (no stacking).</t>
+          <t xml:space="preserve">The features come from a deep network, so the decisions can't be explained. The classifiers are only used one at a time, never combined.</t>
         </is>
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Use a CNN (VGG16) as feature extractor and classify with Random Forest and XGBoost.</t>
+          <t xml:space="preserve">To combine CNN features with classical classifiers for Modi recognition.</t>
         </is>
       </c>
       <c r="M22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">92% accuracy for characters and 93.3% for numerals.</t>
+          <t xml:space="preserve">92% on letters and 93.3% on numerals.</t>
         </is>
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Small dataset (about 5,000 samples).</t>
+          <t xml:space="preserve">Small dataset of around 5,000 images.</t>
         </is>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Features are learned, not handcrafted, so decisions are not interpretable; classifiers are used separately, not stacked; no explainability.</t>
+          <t xml:space="preserve">Handcrafted features, combining the models and explaining the results are all missing. These are exactly what our project adds.</t>
         </is>
       </c>
       <c r="P22" s="4" t="inlineStr">
@@ -1850,12 +1850,12 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Handwritten Modi recognition lags behind other Indian scripts because of writing-style variation.</t>
+          <t xml:space="preserve">Handwritten Modi recognition is behind other Indian scripts because handwriting varies so much.</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Literature review. Tabulates features and classifiers of prior work.</t>
+          <t xml:space="preserve">Short review with a table of earlier methods.</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -1865,7 +1865,7 @@
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Review of Modi handwritten OCR</t>
+          <t xml:space="preserve">Review of Modi handwriting recognition</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
@@ -1875,27 +1875,27 @@
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Short narrative review.</t>
+          <t xml:space="preserve">It's short and mostly descriptive.</t>
         </is>
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Investigate previous research on Modi handwritten character recognition.</t>
+          <t xml:space="preserve">To look at earlier research on recognising handwritten Modi.</t>
         </is>
       </c>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reported classical results vary widely (chain code + BPM 37.5%, KNN 60%, SVM 65%, SVM 99.3% in one study).</t>
+          <t xml:space="preserve">Classical results vary a lot: chain code with BPM 37.5%, KNN 60%, SVM 65%, and one SVM study at 99.3%.</t>
         </is>
       </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Inconsistent datasets and weak features in early work.</t>
+          <t xml:space="preserve">Different datasets and weak features in older work.</t>
         </is>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Short narrative review; shows how weak and inconsistent classical baselines were.</t>
+          <t xml:space="preserve">Shows how weak and inconsistent the older classical baselines were.</t>
         </is>
       </c>
       <c r="P23" s="4" t="inlineStr">
@@ -1928,12 +1928,12 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Modi documents need to be collected, annotated and digitised, but tools for doing so are missing.</t>
+          <t xml:space="preserve">There aren't tools for collecting, labelling and digitising Modi documents.</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toolset: annotation and archiving system, Unicode keyboard, font (MODI-SHAHU), converters.</t>
+          <t xml:space="preserve">Builds an annotation and archiving tool, a Unicode Modi keyboard, a font (MODI-SHAHU) and converters.</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -1943,7 +1943,7 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Modi digitisation: annotation, archiving, Unicode keyboard and font</t>
+          <t xml:space="preserve">Digitising Modi documents and typing in Modi</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
@@ -1953,27 +1953,27 @@
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No OCR component; the authors list OCR as future work.</t>
+          <t xml:space="preserve">There's no OCR part; the authors leave it for future work.</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Provide tools (annotation system, MODI-SHAHU font, keyboard, converters) for Modi preservation.</t>
+          <t xml:space="preserve">To give researchers tools for preserving and digitising Modi.</t>
         </is>
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">A working toolset for digitising Modi; OCR is left as future work.</t>
+          <t xml:space="preserve">A working set of tools, but no recognition.</t>
         </is>
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Script standardisation and community adoption.</t>
+          <t xml:space="preserve">Getting a standard script setup and getting people to use it.</t>
         </is>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No recognition component or evaluation.</t>
+          <t xml:space="preserve">Not a recognition paper, so there's nothing to evaluate.</t>
         </is>
       </c>
       <c r="P24" s="4" t="inlineStr">
@@ -2006,12 +2006,12 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Degraded Modi character images (noise, blur, poor lighting) need effective segmentation before recognition.</t>
+          <t xml:space="preserve">Old Modi images are noisy and blurry, so the letter has to be separated cleanly from the background first.</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Edge detection (Prewitt, Roberts, Canny, Sobel) vs K-means clustering. Image-quality comparison, no classifier.</t>
+          <t xml:space="preserve">Compares edge detection (Prewitt, Roberts, Canny, Sobel) with K-means clustering, using PSNR, MSE and SSIM.</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -2021,7 +2021,7 @@
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pre-processing / segmentation stage of Modi OCR</t>
+          <t xml:space="preserve">Cleaning images before recognition</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
@@ -2031,27 +2031,27 @@
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Works on isolated characters, not on lines or words. No recognition accuracy.</t>
+          <t xml:space="preserve">It only works on single letters, not lines or words, and doesn't report recognition accuracy.</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Compare edge-based (Prewitt, Roberts, Canny, Sobel) and K-means segmentation on Modi characters.</t>
+          <t xml:space="preserve">To find which method separates Modi letters from the background best.</t>
         </is>
       </c>
       <c r="M25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">K-means gives the best quality (PSNR about 50, SSIM about 0.99), especially for numerals.</t>
+          <t xml:space="preserve">K-means worked best (PSNR around 50, SSIM around 0.99), especially for numerals.</t>
         </is>
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Image degradation; segmenting connected strokes.</t>
+          <t xml:space="preserve">Damaged images and strokes that touch each other.</t>
         </is>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Evaluates isolated characters only, not lines or words; no recognition accuracy reported.</t>
+          <t xml:space="preserve">Doesn't show whether better segmentation actually improves recognition.</t>
         </is>
       </c>
       <c r="P25" s="4" t="inlineStr">
@@ -2084,12 +2084,12 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Modi lacks a regular, legible digital font, which limits its use on computers.</t>
+          <t xml:space="preserve">Modi didn't have a clean, regular digital font, so it was hard to use on computers.</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Digital font design (FontForge).</t>
+          <t xml:space="preserve">Designs a new digital Modi font in FontForge.</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
@@ -2099,7 +2099,7 @@
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Typography and digital display of Modi</t>
+          <t xml:space="preserve">Typing and displaying Modi on computers</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
@@ -2109,22 +2109,22 @@
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not a recognition paper.</t>
+          <t xml:space="preserve">It's about font design, not recognition.</t>
         </is>
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Design a new digital Modi font.</t>
+          <t xml:space="preserve">To design a new digital font for Modi.</t>
         </is>
       </c>
       <c r="M26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Produces a regularised digital font (FontForge).</t>
+          <t xml:space="preserve">A regular digital Modi font.</t>
         </is>
       </c>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Non-uniform historical letterforms.</t>
+          <t xml:space="preserve">Historical letter shapes aren't consistent.</t>
         </is>
       </c>
       <c r="O26" s="2" t="inlineStr">
@@ -2162,12 +2162,12 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Building software that recognises cursive Modi characters reliably, regardless of document quality, is difficult.</t>
+          <t xml:space="preserve">It's hard to make software that reliably reads cursive Modi letters from scans of varying quality.</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Grayscale conversion, Otsu binarisation, segmentation. Kohonen neural network (self-organising map).</t>
+          <t xml:space="preserve">Converts to grayscale, uses Otsu thresholding to make it black and white, segments the letters and trains a Kohonen neural network.</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -2187,27 +2187,27 @@
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Only 22 of the characters, 8 training images each, private data.</t>
+          <t xml:space="preserve">Only 22 letters with 8 training images each, on private data.</t>
         </is>
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Recognise 22 Modi characters using Otsu binarisation and a Kohonen neural network.</t>
+          <t xml:space="preserve">To recognise 22 Modi letters using Otsu thresholding and a Kohonen network.</t>
         </is>
       </c>
       <c r="M27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">72.6% recognition for handwritten characters; similar-shaped characters perform worst.</t>
+          <t xml:space="preserve">72.6% on handwritten letters; letters with similar shapes did worst.</t>
         </is>
       </c>
       <c r="N27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Similar character shapes; very few training samples (8 per character).</t>
+          <t xml:space="preserve">Similar-looking letters and very few samples.</t>
         </is>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Only 22 classes and private data; no feature descriptors beyond pixels; no confusion analysis.</t>
+          <t xml:space="preserve">Uses raw pixels with no shape features and doesn't analyse which letters get confused.</t>
         </is>
       </c>
       <c r="P27" s="4" t="inlineStr">
@@ -2240,12 +2240,12 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Handwritten OCR for Indian scripts, and Modi in particular, is still immature.</t>
+          <t xml:space="preserve">Handwriting recognition for Indian scripts, especially Modi, was still at an early stage.</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Literature review. Surveys preprocessing, segmentation, feature extraction, classification.</t>
+          <t xml:space="preserve">Review of preprocessing, segmentation, feature extraction and classification methods for Modi.</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -2265,27 +2265,27 @@
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pre-deep-learning; many cited datasets described as unclear.</t>
+          <t xml:space="preserve">Written before deep learning, and many of the datasets it mentions are unclear.</t>
         </is>
       </c>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Review preprocessing, segmentation, feature extraction and classification work on Modi.</t>
+          <t xml:space="preserve">To review recent work on handwritten Modi OCR.</t>
         </is>
       </c>
       <c r="M28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Early systems report 65.3% to 97% recognition on varied datasets.</t>
+          <t xml:space="preserve">Early systems reported between 65.3% and 97% on different datasets.</t>
         </is>
       </c>
       <c r="N28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Varied writing styles; unclear datasets.</t>
+          <t xml:space="preserve">Different writing styles and unclear data.</t>
         </is>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pre-deep-learning; no common benchmark.</t>
+          <t xml:space="preserve">No common benchmark to compare against.</t>
         </is>
       </c>
       <c r="P28" s="4" t="inlineStr">
@@ -2318,12 +2318,12 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Choosing shape features that describe Modi numerals uniquely and invariantly is key to recognition.</t>
+          <t xml:space="preserve">To recognise Modi digits you need shape features that stay the same even if the digit is moved or rotated.</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hu's seven invariant moments vs Zernike moments (up to 9th order). Distance-based matching.</t>
+          <t xml:space="preserve">Compares Hu's seven moments with Zernike moments (up to order 9), using distance-based matching.</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2333,7 +2333,7 @@
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Recognition of handwritten Modi numerals</t>
+          <t xml:space="preserve">Recognising handwritten Modi digits</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
@@ -2343,27 +2343,27 @@
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Only 100 images and 30 test samples; numerals only. arXiv preprint.</t>
+          <t xml:space="preserve">Only 100 images and 30 test samples, and digits only.</t>
         </is>
       </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Compare Hu's invariant moments with Zernike moments for Modi numerals.</t>
+          <t xml:space="preserve">To compare Hu moments and Zernike moments for Modi digits.</t>
         </is>
       </c>
       <c r="M29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zernike moments 86.66% vs Hu moments 70% (30 test images).</t>
+          <t xml:space="preserve">Zernike moments got 86.66% and Hu moments 70%.</t>
         </is>
       </c>
       <c r="N29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Very small dataset; rotation and position invariance.</t>
+          <t xml:space="preserve">Very small dataset.</t>
         </is>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Only 100 numeral images; descriptors compared, not fused; no letters. Supports using Zernike moments as one descriptor.</t>
+          <t xml:space="preserve">Features are compared but never combined, and letters aren't tested. This is why we use Zernike moments as one of our features.</t>
         </is>
       </c>
       <c r="P29" s="4" t="inlineStr">
@@ -2396,12 +2396,12 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No OCR exists for Modi; its cursive handwriting differs from Devanagari in ways that complicate recognition.</t>
+          <t xml:space="preserve">There was no OCR for Modi, and its cursive handwriting is different from Devanagari in ways that make recognition harder.</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Structural features of Modi characters. Rule-based structural classification (theoretical).</t>
+          <t xml:space="preserve">Theoretical study of Modi letter structure and a rule-based grouping of letters.</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -2411,7 +2411,7 @@
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Theoretical basis for Modi OCR design</t>
+          <t xml:space="preserve">Background for designing a Modi OCR</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
@@ -2421,27 +2421,27 @@
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No implementation.</t>
+          <t xml:space="preserve">No implementation or experiments.</t>
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Analyse Modi characters from a recognition perspective and propose a structural classification.</t>
+          <t xml:space="preserve">To study Modi letters from a recognition point of view.</t>
         </is>
       </c>
       <c r="M30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Identifies the issues that separate Modi from Devanagari and proposes rule-based structural groups.</t>
+          <t xml:space="preserve">Lists what makes Modi different from Devanagari and suggests simple structural groups.</t>
         </is>
       </c>
       <c r="N30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cursive deformation and individual writing styles.</t>
+          <t xml:space="preserve">Cursive strokes and different writing styles.</t>
         </is>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No implementation or experiments.</t>
+          <t xml:space="preserve">Nothing is tested.</t>
         </is>
       </c>
       <c r="P30" s="4" t="inlineStr">
@@ -2474,12 +2474,12 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Modi had no Unicode encoding, so it could not be represented in digital text.</t>
+          <t xml:space="preserve">Modi had no Unicode encoding, so it couldn't be stored as digital text.</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unicode encoding proposal (block U+11600-U+1165F).</t>
+          <t xml:space="preserve">Proposal to add Modi to the Unicode standard (block U+11600 to U+1165F).</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -2489,7 +2489,7 @@
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unicode standard for Modi text</t>
+          <t xml:space="preserve">Unicode support for Modi text</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
@@ -2504,7 +2504,7 @@
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Propose encoding Modi in ISO/IEC 10646 (block U+11600-U+1165F).</t>
+          <t xml:space="preserve">To encode the Modi script in Unicode.</t>
         </is>
       </c>
       <c r="M31" s="2" t="inlineStr">
@@ -2514,12 +2514,12 @@
       </c>
       <c r="N31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Agreeing on a character inventory for a historical script.</t>
+          <t xml:space="preserve">Agreeing on a character list for a historical script.</t>
         </is>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not a recognition paper; serves as the reference inventory for class labels.</t>
+          <t xml:space="preserve">Not about recognition, but it's our reference for which characters exist.</t>
         </is>
       </c>
       <c r="P31" s="4" t="inlineStr">
@@ -2659,17 +2659,17 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Uses the standard public benchmark (46 classes, 90 images each) that most Modi papers report on, and compares a plain CNN with VGG16.</t>
+          <t xml:space="preserve">It uses the public 46-letter dataset (90 images per letter) that most Modi papers test on, and compares a basic CNN with VGG16.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The benchmark size (about 72 training images per class) is our smallest learning-curve point, and its CNN results are our deep-learning reference.</t>
+          <t xml:space="preserve">Their dataset size, about 72 training images per letter, is the starting point for our CNN comparison.</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Their VGG16 shows an 8-point gap between training and validation accuracy. We measure how much data a CNN actually needs, on a fixed test set, instead of reporting one number.</t>
+          <t xml:space="preserve">Their VGG16 does 8 points better on training data than on validation data, so it's overfitting. Instead of one number, we test a CNN at different data sizes on a fixed test set.</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -2707,17 +2707,17 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The strongest recent CNN result on the same benchmark, and it names visually similar characters as the main difficulty.</t>
+          <t xml:space="preserve">It's the best recent CNN result on the same dataset, and it says look-alike letters are the hardest part.</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The idea that the hard part of Modi is telling look-alike characters apart.</t>
+          <t xml:space="preserve">The idea that the real problem in Modi is telling similar letters apart.</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">They describe confused characters but never list them. We list the most confused pairs and use SHAP to show which part of the character separates them.</t>
+          <t xml:space="preserve">They talk about confused letters but never list them. We list the most confused pairs and use SHAP to show which part of the letter tells them apart.</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -2755,17 +2755,17 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Clear published example of deep models overfitting on small Modi data (97% test vs 45% validation, about 21 images per class).</t>
+          <t xml:space="preserve">It's a clear example of a deep model overfitting on small Modi data: 97% on test but 45% on validation, with about 21 images per class.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Motivation for checking data size before trusting deep-learning accuracy on Modi.</t>
+          <t xml:space="preserve">A reason to check how much data a deep model really needs before trusting its accuracy.</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">We keep a single fixed test set and nested training sets, so every accuracy we report is on images the model never saw.</t>
+          <t xml:space="preserve">We keep one fixed test set and only add more training data, so every number we report is on images the model never saw.</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -2803,17 +2803,17 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The only paper that compares classical models (KNN, SVM) and deep models (CNN, VGG16, ResNet) on the same Modi data.</t>
+          <t xml:space="preserve">It's the only paper that tests classical models (KNN, SVM) and deep models (CNN, VGG16, ResNet) on the same Modi data.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The classical-versus-deep comparison itself.</t>
+          <t xml:space="preserve">The idea of comparing classical and deep models directly.</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Their KNN and SVM were given raw pixels, so they had no real chance (75% and 77%). We give the classical models proper handcrafted features and compare at several data sizes.</t>
+          <t xml:space="preserve">Their KNN and SVM got raw pixels, so they scored only 75% and 77%. We give the classical models proper handcrafted features and compare at several data sizes.</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -2851,17 +2851,17 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Closest prior work: it uses Random Forest and XGBoost for Modi characters and numerals.</t>
+          <t xml:space="preserve">It's the closest earlier work: it uses Random Forest and XGBoost for Modi letters and numerals.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Random Forest and XGBoost as classifiers.</t>
+          <t xml:space="preserve">Random Forest and XGBoost as our classifiers.</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">They used VGG16 features (not explainable) and each classifier on its own. We use handcrafted features, combine RF, SVM and XGBoost in a stacking ensemble, and explain every prediction with SHAP.</t>
+          <t xml:space="preserve">They used VGG16 features, which can't be explained, and each classifier on its own. We use handcrafted features, add SVM, combine all three with stacking, and explain each prediction with SHAP.</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -2899,17 +2899,17 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Early Modi recogniser that uses Otsu binarisation, and reports that similar-shaped characters perform worst.</t>
+          <t xml:space="preserve">An early Modi recogniser that uses Otsu thresholding, and it found that similar-shaped letters do worst.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Otsu binarisation as the main preprocessing step.</t>
+          <t xml:space="preserve">Otsu thresholding as our main cleaning step.</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">They used 22 characters with 8 images each and raw pixels. We use all 57 classes, a public dataset and handcrafted descriptors.</t>
+          <t xml:space="preserve">They used 22 letters with 8 images each and raw pixels. We use all 57 classes, a public dataset and handcrafted features.</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
@@ -2947,17 +2947,17 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Shows that Zernike moments describe Modi shapes better than Hu moments (86.7% vs 70%).</t>
+          <t xml:space="preserve">It shows Zernike moments describe Modi shapes better than Hu moments (86.7% vs 70%).</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zernike moments as one of our three descriptors.</t>
+          <t xml:space="preserve">Zernike moments as one of our three features.</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">They tested only 100 digit images with a distance classifier. We fuse Zernike with HOG and LBP on all 57 classes and run an ablation to see what each adds.</t>
+          <t xml:space="preserve">They only tested 100 digit images. We combine Zernike with HOG and LBP on all 57 classes, and test what each feature adds by leaving it out.</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">

</xml_diff>